<commit_message>
PAUSED (task148): stage 4 hardening, patience by call mix, ask pins and devices A4 and B4; stage 3 green, waiting on the reader and judge
The late shift's own callers hold on about two minutes against about ten for the week, so the golden is Erlang A on
the late shift's own censored patience (123.2 s); Erlang C, one patience for every call and every correction of
Erlang C fitted outside the late shift's own hours file May to September. Residual recorded in the design note:
3 of 16 late-shift-at-five scalar correction cells and a free-slope logistic weighted by calls land the set.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task148/golden/late_shift_staffing_fy2028.xlsx
+++ b/task148/golden/late_shift_staffing_fy2028.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="70">
   <si>
     <t>Friday and Saturday late shift (22:00 to 02:00), fiscal 2028: the case for a seasonal fifth call-taker</t>
   </si>
@@ -43,13 +43,13 @@
     <t>Each forecast hour of the late shift is a queue of four call-takers whose callers hang up when they have waited too long (Erlang A), on the Tri-County board's FY2028 forecast for each Friday and Saturday night hour.</t>
   </si>
   <si>
-    <t>Busy time per answered 911 call, answer to Ready, January 2025 to September 2026: 227.0 seconds.</t>
-  </si>
-  <si>
-    <t>Callers' patience: the time all 417,086 911 calls waited, divided by the 7,651 that hung up before an answer: 161.4 seconds. An answered caller's wait only shows that they would have held on at least that long.</t>
-  </si>
-  <si>
-    <t>The standard queue with no hang-ups (Erlang C) would put May to September below 90 per cent; the patience read off the hang-ups' own waits (45.6 seconds) would put no month below it. Neither fits fiscal 2026: see Model check.</t>
+    <t>Busy time per answered 911 call, answer to Ready, January 2025 to September 2026: 226.9 seconds.</t>
+  </si>
+  <si>
+    <t>The agency's callers are not alike. On Friday and Saturday nights from 22:00 they hang up far sooner than at any other time (Model check, patience by segment). The late shift's own callers' patience, the time all 15,814 of its 911 calls waited divided by the 81 that hung up before an answer, is 123.2 seconds; the rest of the week's is 587.7. An answered caller's wait only shows that they would have held on at least that long.</t>
+  </si>
+  <si>
+    <t>The standard queue with no hang-ups (Erlang C), or one patience for every call (576.6 seconds), would put May to September below 90 per cent; the patience read off the late shift's hang-ups' own waits (37.6 seconds) would put no month below it. See Model check.</t>
   </si>
   <si>
     <t>Month</t>
@@ -112,112 +112,121 @@
     <t>Four call-takers on every late-shift night. Compliance as SOP 2.10 measures it: calls answered within 15 seconds over calls presented less those abandoned within 5 seconds; each night counted in the month it starts.</t>
   </si>
   <si>
-    <t>Fiscal 2026 predicted from January to June 2025 (busy time 226.5 s, patience 157.5 s, hang-ups' own wait 45.4 s), every hour on its own call-takers and calls</t>
+    <t>Fiscal 2026 predicted from January to June 2025 (busy time 226.4 s; patience 180.3 s on the late shift, 602.5 s at other hours, 594.2 s for every call together), every hour on its own call-takers and calls</t>
+  </si>
+  <si>
+    <t>Hours</t>
+  </si>
+  <si>
+    <t>Calls</t>
   </si>
   <si>
     <t>Observed compliance (%)</t>
   </si>
   <si>
-    <t>Erlang A, patience over every wait (%)</t>
+    <t>Observed hang-ups (% of calls)</t>
+  </si>
+  <si>
+    <t>Erlang A, each segment's patience (%)</t>
+  </si>
+  <si>
+    <t>Hang-ups (% of calls)</t>
+  </si>
+  <si>
+    <t>Erlang A, one patience (%)</t>
   </si>
   <si>
     <t>Erlang C (%)</t>
   </si>
   <si>
-    <t>Erlang A, hang-ups' own waits (%)</t>
-  </si>
-  <si>
-    <t>Observed hang-ups (%)</t>
-  </si>
-  <si>
-    <t>Erlang A hang-ups (%)</t>
-  </si>
-  <si>
-    <t>Hang-ups' own waits: hang-ups (%)</t>
-  </si>
-  <si>
-    <t>Jul 2025</t>
-  </si>
-  <si>
-    <t>Aug 2025</t>
-  </si>
-  <si>
-    <t>Sep 2025</t>
-  </si>
-  <si>
-    <t>Oct 2025</t>
-  </si>
-  <si>
-    <t>Nov 2025</t>
-  </si>
-  <si>
-    <t>Dec 2025</t>
-  </si>
-  <si>
-    <t>Jan 2026</t>
-  </si>
-  <si>
-    <t>Feb 2026</t>
-  </si>
-  <si>
-    <t>Mar 2026</t>
-  </si>
-  <si>
-    <t>Apr 2026</t>
+    <t>Friday and Saturday late shift</t>
+  </si>
+  <si>
+    <t>Every other hour</t>
+  </si>
+  <si>
+    <t>The whole floor</t>
+  </si>
+  <si>
+    <t>Patience by segment, January 2025 to September 2026</t>
+  </si>
+  <si>
+    <t>911 calls</t>
+  </si>
+  <si>
+    <t>Hung up before an answer</t>
+  </si>
+  <si>
+    <t>Total waiting time (s)</t>
+  </si>
+  <si>
+    <t>Patience (s)</t>
+  </si>
+  <si>
+    <t>Friday and Saturday nights, 22:00 to 02:00 (the late shift)</t>
+  </si>
+  <si>
+    <t>Friday and Saturday nights, 02:00 to 06:00</t>
+  </si>
+  <si>
+    <t>Other nights, 22:00 to 06:00</t>
+  </si>
+  <si>
+    <t>06:00 to 18:00</t>
+  </si>
+  <si>
+    <t>18:00 to 22:00</t>
+  </si>
+  <si>
+    <t>Patience is the total time the segment's calls waited, answered or not, over the calls that hung up: an answered call's wait is time its caller held on.</t>
+  </si>
+  <si>
+    <t>Quarter</t>
+  </si>
+  <si>
+    <t>Wireless 911 calls placed from Halvorsen Township that reached the agency</t>
+  </si>
+  <si>
+    <t>Of them, transferred to Wexley County Emergency Communications</t>
+  </si>
+  <si>
+    <t>Q1 (July to September 2025)</t>
+  </si>
+  <si>
+    <t>Q2 (October to December 2025)</t>
+  </si>
+  <si>
+    <t>Q3 (January to March 2026)</t>
+  </si>
+  <si>
+    <t>Q4 (April to June 2026)</t>
+  </si>
+  <si>
+    <t>Placed by each call's last handset location in the township boundary, answered or not, the backup centre's records found by the call's incident identifier; transfers to either of Wexley's PSAP URIs in the ESInet directory.</t>
+  </si>
+  <si>
+    <t>Abandoned 911 calls</t>
+  </si>
+  <si>
+    <t>Dialled back within two minutes</t>
+  </si>
+  <si>
+    <t>Share (%)</t>
+  </si>
+  <si>
+    <t>January 2026</t>
+  </si>
+  <si>
+    <t>February 2026</t>
+  </si>
+  <si>
+    <t>March 2026</t>
+  </si>
+  <si>
+    <t>April 2026</t>
   </si>
   <si>
     <t>May 2026</t>
-  </si>
-  <si>
-    <t>Jun 2026</t>
-  </si>
-  <si>
-    <t>Fiscal 2026</t>
-  </si>
-  <si>
-    <t>Quarter</t>
-  </si>
-  <si>
-    <t>Wireless 911 calls placed from Halvorsen Township that reached the agency</t>
-  </si>
-  <si>
-    <t>Of them, transferred to Wexley County Emergency Communications</t>
-  </si>
-  <si>
-    <t>Q1 (July to September 2025)</t>
-  </si>
-  <si>
-    <t>Q2 (October to December 2025)</t>
-  </si>
-  <si>
-    <t>Q3 (January to March 2026)</t>
-  </si>
-  <si>
-    <t>Q4 (April to June 2026)</t>
-  </si>
-  <si>
-    <t>Placed by each call's handset location in the township boundary, answered or not; transfers to either of Wexley's PSAP URIs in the ESInet directory.</t>
-  </si>
-  <si>
-    <t>Abandoned 911 calls</t>
-  </si>
-  <si>
-    <t>Dialled back within two minutes</t>
-  </si>
-  <si>
-    <t>Share (%)</t>
-  </si>
-  <si>
-    <t>January 2026</t>
-  </si>
-  <si>
-    <t>February 2026</t>
-  </si>
-  <si>
-    <t>March 2026</t>
-  </si>
-  <si>
-    <t>April 2026</t>
   </si>
   <si>
     <t>June 2026</t>
@@ -292,7 +301,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -307,10 +316,14 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -715,7 +728,7 @@
         <v>10</v>
       </c>
       <c r="C2" s="6">
-        <v>1296</v>
+        <v>1323</v>
       </c>
       <c r="D2" s="5">
         <v>88</v>
@@ -732,7 +745,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="6">
-        <v>1007</v>
+        <v>1027</v>
       </c>
       <c r="D3" s="5">
         <v>89</v>
@@ -749,7 +762,7 @@
         <v>8</v>
       </c>
       <c r="C4" s="7">
-        <v>926</v>
+        <v>942</v>
       </c>
       <c r="D4">
         <v>91</v>
@@ -766,7 +779,7 @@
         <v>10</v>
       </c>
       <c r="C5" s="7">
-        <v>1062</v>
+        <v>1080</v>
       </c>
       <c r="D5">
         <v>93</v>
@@ -783,7 +796,7 @@
         <v>8</v>
       </c>
       <c r="C6" s="7">
-        <v>825</v>
+        <v>837</v>
       </c>
       <c r="D6">
         <v>94</v>
@@ -800,7 +813,7 @@
         <v>9</v>
       </c>
       <c r="C7" s="7">
-        <v>960</v>
+        <v>975</v>
       </c>
       <c r="D7">
         <v>93</v>
@@ -817,7 +830,7 @@
         <v>9</v>
       </c>
       <c r="C8" s="7">
-        <v>902</v>
+        <v>916</v>
       </c>
       <c r="D8">
         <v>94</v>
@@ -834,7 +847,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="7">
-        <v>756</v>
+        <v>767</v>
       </c>
       <c r="D9">
         <v>95</v>
@@ -851,7 +864,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="7">
-        <v>898</v>
+        <v>912</v>
       </c>
       <c r="D10">
         <v>94</v>
@@ -868,7 +881,7 @@
         <v>9</v>
       </c>
       <c r="C11" s="7">
-        <v>959</v>
+        <v>975</v>
       </c>
       <c r="D11">
         <v>93</v>
@@ -885,7 +898,7 @@
         <v>8</v>
       </c>
       <c r="C12" s="7">
-        <v>929</v>
+        <v>945</v>
       </c>
       <c r="D12">
         <v>91</v>
@@ -902,7 +915,7 @@
         <v>9</v>
       </c>
       <c r="C13" s="6">
-        <v>1131</v>
+        <v>1153</v>
       </c>
       <c r="D13" s="5">
         <v>89</v>
@@ -923,386 +936,251 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EABECF4A-E05D-56DB-827F-08CAA5EC9E49}">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="44.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" customWidth="1"/>
     <col min="5" max="5" width="20.7109375" customWidth="1"/>
     <col min="6" max="6" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" customWidth="1"/>
+    <col min="7" max="7" width="18.7109375" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="4" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="B3" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="C3" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="D3" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="E3" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="F3" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="G3" s="8" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="H3" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="8">
-        <v>92.40000000000001</v>
-      </c>
-      <c r="C4" s="8">
-        <v>92.7</v>
-      </c>
-      <c r="D4" s="8">
-        <v>89.59999999999999</v>
-      </c>
-      <c r="E4" s="8">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="9">
+        <v>8921</v>
+      </c>
+      <c r="C4" s="10">
+        <v>99.09999999999999</v>
+      </c>
+      <c r="D4" s="11">
+        <v>0.46</v>
+      </c>
+      <c r="E4" s="10">
+        <v>98.90000000000001</v>
+      </c>
+      <c r="F4" s="11">
+        <v>0.34</v>
+      </c>
+      <c r="G4" s="10">
+        <v>98.8</v>
+      </c>
+      <c r="H4" s="11">
+        <v>0.14</v>
+      </c>
+      <c r="I4" s="10">
+        <v>98.7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="7">
+        <v>227132</v>
+      </c>
+      <c r="C5" s="12">
         <v>94.5</v>
       </c>
-      <c r="F4" s="9">
-        <v>2.74</v>
-      </c>
-      <c r="G4" s="9">
-        <v>2.72</v>
-      </c>
-      <c r="H4" s="9">
-        <v>4.25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="8">
-        <v>92.90000000000001</v>
-      </c>
-      <c r="C5" s="8">
-        <v>93.2</v>
-      </c>
-      <c r="D5" s="8">
-        <v>90.5</v>
-      </c>
-      <c r="E5" s="8">
-        <v>94.90000000000001</v>
-      </c>
-      <c r="F5" s="9">
-        <v>2.46</v>
-      </c>
-      <c r="G5" s="9">
-        <v>2.53</v>
-      </c>
-      <c r="H5" s="9">
-        <v>3.96</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D5" s="13">
+        <v>0.78</v>
+      </c>
+      <c r="E5" s="12">
+        <v>94.3</v>
+      </c>
+      <c r="F5" s="13">
+        <v>0.78</v>
+      </c>
+      <c r="G5" s="12">
+        <v>94.3</v>
+      </c>
+      <c r="H5" s="13">
+        <v>0.79</v>
+      </c>
+      <c r="I5" s="12">
+        <v>93.59999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="8">
-        <v>95.09999999999999</v>
-      </c>
-      <c r="C6" s="8">
-        <v>95.2</v>
-      </c>
-      <c r="D6" s="8">
-        <v>93.7</v>
-      </c>
-      <c r="E6" s="8">
-        <v>96.3</v>
-      </c>
-      <c r="F6" s="9">
-        <v>1.71</v>
-      </c>
-      <c r="G6" s="9">
-        <v>1.73</v>
-      </c>
-      <c r="H6" s="9">
-        <v>2.84</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="8">
-        <v>96.40000000000001</v>
-      </c>
-      <c r="C7" s="8">
-        <v>96.2</v>
-      </c>
-      <c r="D7" s="8">
-        <v>95</v>
-      </c>
-      <c r="E7" s="8">
-        <v>97</v>
-      </c>
-      <c r="F7" s="9">
-        <v>1.27</v>
-      </c>
-      <c r="G7" s="9">
-        <v>1.43</v>
-      </c>
-      <c r="H7" s="9">
-        <v>2.34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B6" s="7">
+        <v>236053</v>
+      </c>
+      <c r="C6" s="12">
+        <v>94.7</v>
+      </c>
+      <c r="D6" s="13">
+        <v>0.77</v>
+      </c>
+      <c r="E6" s="12">
+        <v>94.5</v>
+      </c>
+      <c r="F6" s="13">
+        <v>0.77</v>
+      </c>
+      <c r="G6" s="12">
+        <v>94.5</v>
+      </c>
+      <c r="H6" s="13">
+        <v>0.77</v>
+      </c>
+      <c r="I6" s="12">
+        <v>93.8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="8">
-        <v>96.2</v>
-      </c>
-      <c r="C8" s="8">
-        <v>96.5</v>
-      </c>
-      <c r="D8" s="8">
-        <v>95.40000000000001</v>
-      </c>
-      <c r="E8" s="8">
-        <v>97.2</v>
-      </c>
-      <c r="F8" s="9">
-        <v>1.5</v>
-      </c>
-      <c r="G8" s="9">
-        <v>1.3</v>
-      </c>
-      <c r="H8" s="9">
-        <v>2.15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="8">
-        <v>95.8</v>
-      </c>
-      <c r="C9" s="8">
-        <v>96.3</v>
-      </c>
-      <c r="D9" s="8">
-        <v>95.09999999999999</v>
-      </c>
-      <c r="E9" s="8">
-        <v>97.09999999999999</v>
-      </c>
-      <c r="F9" s="9">
-        <v>1.45</v>
-      </c>
-      <c r="G9" s="9">
-        <v>1.36</v>
-      </c>
-      <c r="H9" s="9">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="C10" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="8">
-        <v>96.8</v>
-      </c>
-      <c r="C10" s="8">
-        <v>96.8</v>
-      </c>
-      <c r="D10" s="8">
-        <v>95.90000000000001</v>
-      </c>
-      <c r="E10" s="8">
-        <v>97.5</v>
-      </c>
-      <c r="F10" s="9">
-        <v>1.17</v>
-      </c>
-      <c r="G10" s="9">
-        <v>1.17</v>
-      </c>
-      <c r="H10" s="9">
-        <v>1.96</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D10" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" s="8">
-        <v>97.59999999999999</v>
-      </c>
-      <c r="C11" s="8">
-        <v>97.09999999999999</v>
-      </c>
-      <c r="D11" s="8">
-        <v>96.3</v>
-      </c>
-      <c r="E11" s="8">
-        <v>97.7</v>
-      </c>
-      <c r="F11" s="9">
-        <v>0.9</v>
-      </c>
-      <c r="G11" s="9">
-        <v>1.06</v>
-      </c>
-      <c r="H11" s="9">
-        <v>1.78</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="B11" s="7">
+        <v>15814</v>
+      </c>
+      <c r="C11" s="7">
+        <v>81</v>
+      </c>
+      <c r="D11" s="7">
+        <v>9976</v>
+      </c>
+      <c r="E11" s="12">
+        <v>123.2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>45</v>
-      </c>
-      <c r="B12" s="8">
-        <v>96.2</v>
-      </c>
-      <c r="C12" s="8">
-        <v>96.59999999999999</v>
-      </c>
-      <c r="D12" s="8">
-        <v>95.7</v>
-      </c>
-      <c r="E12" s="8">
-        <v>97.40000000000001</v>
-      </c>
-      <c r="F12" s="9">
-        <v>1.34</v>
-      </c>
-      <c r="G12" s="9">
-        <v>1.23</v>
-      </c>
-      <c r="H12" s="9">
-        <v>2.04</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+      <c r="B12" s="7">
+        <v>7419</v>
+      </c>
+      <c r="C12" s="7">
+        <v>115</v>
+      </c>
+      <c r="D12" s="7">
+        <v>13698</v>
+      </c>
+      <c r="E12" s="12">
+        <v>119.1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" s="8">
-        <v>96.59999999999999</v>
-      </c>
-      <c r="C13" s="8">
-        <v>96.40000000000001</v>
-      </c>
-      <c r="D13" s="8">
-        <v>95.3</v>
-      </c>
-      <c r="E13" s="8">
-        <v>97.2</v>
-      </c>
-      <c r="F13" s="9">
-        <v>1.19</v>
-      </c>
-      <c r="G13" s="9">
-        <v>1.31</v>
-      </c>
-      <c r="H13" s="9">
-        <v>2.19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="B13" s="7">
+        <v>49524</v>
+      </c>
+      <c r="C13" s="7">
+        <v>253</v>
+      </c>
+      <c r="D13" s="7">
+        <v>133902</v>
+      </c>
+      <c r="E13" s="12">
+        <v>529.3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>47</v>
-      </c>
-      <c r="B14" s="8">
-        <v>95.3</v>
-      </c>
-      <c r="C14" s="8">
-        <v>95.09999999999999</v>
-      </c>
-      <c r="D14" s="8">
-        <v>93.5</v>
-      </c>
-      <c r="E14" s="8">
-        <v>96.2</v>
-      </c>
-      <c r="F14" s="9">
-        <v>1.81</v>
-      </c>
-      <c r="G14" s="9">
-        <v>1.79</v>
-      </c>
-      <c r="H14" s="9">
-        <v>2.91</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+      <c r="B14" s="7">
+        <v>247066</v>
+      </c>
+      <c r="C14" s="7">
+        <v>1384</v>
+      </c>
+      <c r="D14" s="7">
+        <v>869506</v>
+      </c>
+      <c r="E14" s="12">
+        <v>628.3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B15" s="8">
-        <v>93.5</v>
-      </c>
-      <c r="C15" s="8">
-        <v>93.5</v>
-      </c>
-      <c r="D15" s="8">
-        <v>91.09999999999999</v>
-      </c>
-      <c r="E15" s="8">
-        <v>95.09999999999999</v>
-      </c>
-      <c r="F15" s="9">
-        <v>2.27</v>
-      </c>
-      <c r="G15" s="9">
-        <v>2.41</v>
-      </c>
-      <c r="H15" s="9">
-        <v>3.82</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B16" s="10">
-        <v>95.2</v>
-      </c>
-      <c r="C16" s="10">
-        <v>95.3</v>
-      </c>
-      <c r="D16" s="10">
-        <v>93.7</v>
-      </c>
-      <c r="E16" s="10">
-        <v>96.40000000000001</v>
-      </c>
-      <c r="F16" s="11">
-        <v>1.71</v>
-      </c>
-      <c r="G16" s="11">
-        <v>1.73</v>
-      </c>
-      <c r="H16" s="11">
-        <v>2.79</v>
+        <v>50</v>
+      </c>
+      <c r="B15" s="7">
+        <v>96798</v>
+      </c>
+      <c r="C15" s="7">
+        <v>1574</v>
+      </c>
+      <c r="D15" s="7">
+        <v>937479</v>
+      </c>
+      <c r="E15" s="12">
+        <v>595.6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1321,63 +1199,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="C1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>52</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B2" s="7">
-        <v>1473</v>
+        <v>1475</v>
       </c>
       <c r="C2" s="7">
-        <v>1304</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B3" s="7">
-        <v>1249</v>
+        <v>1243</v>
       </c>
       <c r="C3" s="7">
-        <v>1126</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B4" s="7">
         <v>1104</v>
       </c>
       <c r="C4" s="7">
-        <v>1001</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B5" s="7">
-        <v>1265</v>
+        <v>1253</v>
       </c>
       <c r="C5" s="7">
-        <v>1154</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1401,102 +1279,102 @@
         <v>9</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B2">
-        <v>213</v>
+        <v>96</v>
       </c>
       <c r="C2">
-        <v>117</v>
-      </c>
-      <c r="D2" s="8">
-        <v>54.9</v>
+        <v>53</v>
+      </c>
+      <c r="D2" s="12">
+        <v>55.2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B3">
-        <v>141</v>
+        <v>51</v>
       </c>
       <c r="C3">
-        <v>78</v>
-      </c>
-      <c r="D3" s="8">
-        <v>55.3</v>
+        <v>23</v>
+      </c>
+      <c r="D3" s="12">
+        <v>45.1</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B4">
+        <v>111</v>
+      </c>
+      <c r="C4">
         <v>63</v>
       </c>
-      <c r="B4">
-        <v>245</v>
-      </c>
-      <c r="C4">
-        <v>126</v>
-      </c>
-      <c r="D4" s="8">
-        <v>51.4</v>
+      <c r="D4" s="12">
+        <v>56.8</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B5">
-        <v>220</v>
+        <v>97</v>
       </c>
       <c r="C5">
-        <v>118</v>
-      </c>
-      <c r="D5" s="8">
-        <v>53.6</v>
+        <v>51</v>
+      </c>
+      <c r="D5" s="12">
+        <v>52.6</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="B6">
-        <v>379</v>
+        <v>187</v>
       </c>
       <c r="C6">
-        <v>183</v>
-      </c>
-      <c r="D6" s="8">
-        <v>48.3</v>
+        <v>94</v>
+      </c>
+      <c r="D6" s="12">
+        <v>50.3</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B7">
-        <v>496</v>
+        <v>216</v>
       </c>
       <c r="C7">
-        <v>256</v>
-      </c>
-      <c r="D7" s="8">
-        <v>51.6</v>
+        <v>111</v>
+      </c>
+      <c r="D7" s="12">
+        <v>51.4</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>